<commit_message>
[design] MG996R v1.0 완료: 14축 전부 MG996R, 1.5배 어셈블리·BOM·MJCF·검증
- hobby_layout 등에 MD_VARIANT=mg996r: 머리 yaw/roll MG996R, 머리 yaw 6706ZZ, 머리 셸 나사 3곳
- 배치 간섭 0, 메시 간섭 새 간섭 0, 관절 14/14, STAND 유지 (무릎 26%)
- hobby_joints_check.py (Fusion +20도 실측 vs MJCF), BOM 스크립트 판별 출력

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QbojE4FFgsiDig29qW2GQW
</commit_message>
<xml_diff>
--- a/cad/redesign/hobby_servo/v1.0/BOM_hobby_servo_v1.0.xlsx
+++ b/cad/redesign/hobby_servo/v1.0/BOM_hobby_servo_v1.0.xlsx
@@ -497,7 +497,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Microduck 일반 서보 v1.0 BOM — 어셈블리 1_microduck_hobby_servo_v1.0 (Fusion 개인/microduck_hobby_servo_v1.0)</t>
+          <t>Microduck hobby_servo v1.0 BOM — 어셈블리 1_microduck_hobby_servo_v1.0 (Fusion 개인/microduck_hobby_servo_v1.0)</t>
         </is>
       </c>
     </row>
@@ -2039,7 +2039,7 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>얇은 볼베어링 30×37×4 (고관절 yaw 혼 둘레)</t>
+          <t>얇은 볼베어링 30×37×4 (yaw 관절 혼 둘레)</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">

</xml_diff>